<commit_message>
updated roll of honour css
</commit_message>
<xml_diff>
--- a/excels/awards and honours.xlsx
+++ b/excels/awards and honours.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26BEDFB0-F500-406E-98C6-BA36C7FEED23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A79A6A02-AD38-449C-B019-32E6DA6B4CDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Roll of honours" sheetId="1" r:id="rId1"/>
@@ -614,10 +614,10 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>1970</v>
+        <v>2024</v>
       </c>
       <c r="C2" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -625,10 +625,10 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1972</v>
+        <v>2023</v>
       </c>
       <c r="C3" t="s">
-        <v>3</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -636,10 +636,10 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>1973</v>
+        <v>2022</v>
       </c>
       <c r="C4" t="s">
-        <v>4</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -647,10 +647,10 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>1974</v>
+        <v>2021</v>
       </c>
       <c r="C5" t="s">
-        <v>5</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -658,10 +658,10 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>1975</v>
+        <v>2020</v>
       </c>
       <c r="C6" t="s">
-        <v>6</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -669,10 +669,10 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>1976</v>
+        <v>2019</v>
       </c>
       <c r="C7" t="s">
-        <v>7</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -680,10 +680,10 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>1977</v>
+        <v>2018</v>
       </c>
       <c r="C8" t="s">
-        <v>8</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -691,10 +691,10 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>1978</v>
+        <v>2017</v>
       </c>
       <c r="C9" t="s">
-        <v>9</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -702,10 +702,10 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>1979</v>
+        <v>2016</v>
       </c>
       <c r="C10" t="s">
-        <v>10</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -713,10 +713,10 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>1980</v>
+        <v>2015</v>
       </c>
       <c r="C11" t="s">
-        <v>11</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -724,10 +724,10 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>1981</v>
+        <v>2014</v>
       </c>
       <c r="C12" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -735,10 +735,10 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>1982</v>
+        <v>2013</v>
       </c>
       <c r="C13" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -746,10 +746,10 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>1983</v>
+        <v>2012</v>
       </c>
       <c r="C14" t="s">
-        <v>14</v>
+        <v>44</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -757,10 +757,10 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>1984</v>
+        <v>2011</v>
       </c>
       <c r="C15" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -768,10 +768,10 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>1985</v>
+        <v>2010</v>
       </c>
       <c r="C16" t="s">
-        <v>16</v>
+        <v>42</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -779,10 +779,10 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>1986</v>
+        <v>2009</v>
       </c>
       <c r="C17" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -790,10 +790,10 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>1987</v>
+        <v>2008</v>
       </c>
       <c r="C18" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -801,10 +801,10 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>1988</v>
+        <v>2007</v>
       </c>
       <c r="C19" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -812,10 +812,10 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>1989</v>
+        <v>2006</v>
       </c>
       <c r="C20" t="s">
-        <v>20</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -823,10 +823,10 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>1990</v>
+        <v>2005</v>
       </c>
       <c r="C21" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -834,10 +834,10 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>1991</v>
+        <v>2004</v>
       </c>
       <c r="C22" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -845,10 +845,10 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>1992</v>
+        <v>2003</v>
       </c>
       <c r="C23" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -856,10 +856,10 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>1993</v>
+        <v>2002</v>
       </c>
       <c r="C24" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -867,10 +867,10 @@
         <v>24</v>
       </c>
       <c r="B25">
-        <v>1994</v>
+        <v>2001</v>
       </c>
       <c r="C25" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -878,10 +878,10 @@
         <v>25</v>
       </c>
       <c r="B26">
-        <v>1995</v>
+        <v>2000</v>
       </c>
       <c r="C26" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -889,10 +889,10 @@
         <v>26</v>
       </c>
       <c r="B27">
-        <v>1996</v>
+        <v>1999</v>
       </c>
       <c r="C27" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -900,10 +900,10 @@
         <v>27</v>
       </c>
       <c r="B28">
-        <v>1997</v>
+        <v>1998</v>
       </c>
       <c r="C28" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -911,10 +911,10 @@
         <v>28</v>
       </c>
       <c r="B29">
-        <v>1998</v>
+        <v>1997</v>
       </c>
       <c r="C29" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -922,10 +922,10 @@
         <v>29</v>
       </c>
       <c r="B30">
-        <v>1999</v>
+        <v>1996</v>
       </c>
       <c r="C30" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -933,10 +933,10 @@
         <v>30</v>
       </c>
       <c r="B31">
-        <v>2000</v>
+        <v>1995</v>
       </c>
       <c r="C31" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -944,10 +944,10 @@
         <v>31</v>
       </c>
       <c r="B32">
-        <v>2001</v>
+        <v>1994</v>
       </c>
       <c r="C32" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -955,10 +955,10 @@
         <v>32</v>
       </c>
       <c r="B33">
-        <v>2002</v>
+        <v>1993</v>
       </c>
       <c r="C33" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -966,10 +966,10 @@
         <v>33</v>
       </c>
       <c r="B34">
-        <v>2003</v>
+        <v>1992</v>
       </c>
       <c r="C34" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -977,10 +977,10 @@
         <v>34</v>
       </c>
       <c r="B35">
-        <v>2004</v>
+        <v>1991</v>
       </c>
       <c r="C35" t="s">
-        <v>36</v>
+        <v>22</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -988,10 +988,10 @@
         <v>35</v>
       </c>
       <c r="B36">
-        <v>2005</v>
+        <v>1990</v>
       </c>
       <c r="C36" t="s">
-        <v>37</v>
+        <v>21</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -999,10 +999,10 @@
         <v>36</v>
       </c>
       <c r="B37">
-        <v>2006</v>
+        <v>1989</v>
       </c>
       <c r="C37" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -1010,10 +1010,10 @@
         <v>37</v>
       </c>
       <c r="B38">
-        <v>2007</v>
+        <v>1988</v>
       </c>
       <c r="C38" t="s">
-        <v>39</v>
+        <v>19</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
@@ -1021,10 +1021,10 @@
         <v>38</v>
       </c>
       <c r="B39">
-        <v>2008</v>
+        <v>1987</v>
       </c>
       <c r="C39" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -1032,10 +1032,10 @@
         <v>39</v>
       </c>
       <c r="B40">
-        <v>2009</v>
+        <v>1986</v>
       </c>
       <c r="C40" t="s">
-        <v>41</v>
+        <v>17</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
@@ -1043,10 +1043,10 @@
         <v>40</v>
       </c>
       <c r="B41">
-        <v>2010</v>
+        <v>1985</v>
       </c>
       <c r="C41" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
@@ -1054,10 +1054,10 @@
         <v>41</v>
       </c>
       <c r="B42">
-        <v>2011</v>
+        <v>1984</v>
       </c>
       <c r="C42" t="s">
-        <v>43</v>
+        <v>15</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
@@ -1065,10 +1065,10 @@
         <v>42</v>
       </c>
       <c r="B43">
-        <v>2012</v>
+        <v>1983</v>
       </c>
       <c r="C43" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -1076,10 +1076,10 @@
         <v>43</v>
       </c>
       <c r="B44">
-        <v>2013</v>
+        <v>1982</v>
       </c>
       <c r="C44" t="s">
-        <v>45</v>
+        <v>13</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -1087,10 +1087,10 @@
         <v>44</v>
       </c>
       <c r="B45">
-        <v>2014</v>
+        <v>1981</v>
       </c>
       <c r="C45" t="s">
-        <v>46</v>
+        <v>12</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
@@ -1098,10 +1098,10 @@
         <v>45</v>
       </c>
       <c r="B46">
-        <v>2015</v>
+        <v>1980</v>
       </c>
       <c r="C46" t="s">
-        <v>47</v>
+        <v>11</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
@@ -1109,10 +1109,10 @@
         <v>46</v>
       </c>
       <c r="B47">
-        <v>2016</v>
+        <v>1979</v>
       </c>
       <c r="C47" t="s">
-        <v>48</v>
+        <v>10</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
@@ -1120,10 +1120,10 @@
         <v>47</v>
       </c>
       <c r="B48">
-        <v>2017</v>
+        <v>1978</v>
       </c>
       <c r="C48" t="s">
-        <v>49</v>
+        <v>9</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -1131,10 +1131,10 @@
         <v>48</v>
       </c>
       <c r="B49">
-        <v>2018</v>
+        <v>1977</v>
       </c>
       <c r="C49" t="s">
-        <v>50</v>
+        <v>8</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -1142,10 +1142,10 @@
         <v>49</v>
       </c>
       <c r="B50">
-        <v>2019</v>
+        <v>1976</v>
       </c>
       <c r="C50" t="s">
-        <v>51</v>
+        <v>7</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -1153,10 +1153,10 @@
         <v>50</v>
       </c>
       <c r="B51">
-        <v>2020</v>
+        <v>1975</v>
       </c>
       <c r="C51" t="s">
-        <v>52</v>
+        <v>6</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
@@ -1164,10 +1164,10 @@
         <v>51</v>
       </c>
       <c r="B52">
-        <v>2021</v>
+        <v>1974</v>
       </c>
       <c r="C52" t="s">
-        <v>53</v>
+        <v>5</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
@@ -1175,10 +1175,10 @@
         <v>52</v>
       </c>
       <c r="B53">
-        <v>2022</v>
+        <v>1973</v>
       </c>
       <c r="C53" t="s">
-        <v>54</v>
+        <v>4</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
@@ -1186,10 +1186,10 @@
         <v>53</v>
       </c>
       <c r="B54">
-        <v>2023</v>
+        <v>1972</v>
       </c>
       <c r="C54" t="s">
-        <v>55</v>
+        <v>3</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
@@ -1197,13 +1197,16 @@
         <v>54</v>
       </c>
       <c r="B55">
-        <v>2024</v>
+        <v>1970</v>
       </c>
       <c r="C55" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C55">
+    <sortCondition descending="1" ref="B2:B55"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1229,156 +1232,156 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>2010</v>
+        <v>2022</v>
       </c>
       <c r="B2" t="s">
         <v>59</v>
       </c>
       <c r="C2" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>2011</v>
+        <v>2022</v>
       </c>
       <c r="B3" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C3" t="s">
-        <v>42</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>2012</v>
+        <v>2022</v>
       </c>
       <c r="B4" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C4" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>2013</v>
+        <v>2021</v>
       </c>
       <c r="B5" t="s">
         <v>59</v>
       </c>
       <c r="C5" t="s">
-        <v>61</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>2014</v>
+        <v>2021</v>
       </c>
       <c r="B6" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C6" t="s">
-        <v>46</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>2015</v>
+        <v>2021</v>
       </c>
       <c r="B7" t="s">
-        <v>82</v>
+        <v>65</v>
       </c>
       <c r="C7" t="s">
-        <v>62</v>
+        <v>75</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>2015</v>
+        <v>2020</v>
       </c>
       <c r="B8" t="s">
-        <v>81</v>
+        <v>59</v>
       </c>
       <c r="C8" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>2015</v>
+        <v>2020</v>
       </c>
       <c r="B9" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C9" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>2016</v>
+        <v>2020</v>
       </c>
       <c r="B10" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C10" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>2016</v>
+        <v>2019</v>
       </c>
       <c r="B11" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C11" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>2016</v>
+        <v>2019</v>
       </c>
       <c r="B12" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C12" t="s">
-        <v>68</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>2017</v>
+        <v>2019</v>
       </c>
       <c r="B13" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C13" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="B14" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="B15" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C15" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -1386,167 +1389,170 @@
         <v>2018</v>
       </c>
       <c r="B16" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C16" t="s">
-        <v>71</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>2018</v>
+        <v>2017</v>
       </c>
       <c r="B17" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C17" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>2018</v>
+        <v>2017</v>
       </c>
       <c r="B18" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C18" t="s">
-        <v>49</v>
+        <v>70</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19">
-        <v>2019</v>
+        <v>2017</v>
       </c>
       <c r="B19" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C19" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="B20" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C20" t="s">
-        <v>51</v>
+        <v>67</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="B21" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C21" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22">
-        <v>2020</v>
+        <v>2016</v>
       </c>
       <c r="B22" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C22" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23">
-        <v>2020</v>
+        <v>2015</v>
       </c>
       <c r="B23" t="s">
-        <v>63</v>
+        <v>82</v>
       </c>
       <c r="C23" t="s">
-        <v>76</v>
+        <v>62</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24">
-        <v>2020</v>
+        <v>2015</v>
       </c>
       <c r="B24" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="C24" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25">
-        <v>2021</v>
+        <v>2015</v>
       </c>
       <c r="B25" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C25" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26">
-        <v>2021</v>
+        <v>2014</v>
       </c>
       <c r="B26" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C26" t="s">
-        <v>79</v>
+        <v>46</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27">
-        <v>2021</v>
+        <v>2013</v>
       </c>
       <c r="B27" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="C27" t="s">
-        <v>75</v>
+        <v>61</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28">
-        <v>2022</v>
+        <v>2012</v>
       </c>
       <c r="B28" t="s">
         <v>59</v>
       </c>
       <c r="C28" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29">
-        <v>2022</v>
+        <v>2011</v>
       </c>
       <c r="B29" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C29" t="s">
-        <v>80</v>
+        <v>42</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30">
-        <v>2022</v>
+        <v>2010</v>
       </c>
       <c r="B30" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="C30" t="s">
-        <v>83</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C30">
+    <sortCondition descending="1" ref="A2:A30"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>